<commit_message>
update description and update array 441aa88e99de9763eead322de81cdd70aa57578e
</commit_message>
<xml_diff>
--- a/ig/nr-add-nos-generate-profil-table/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
+++ b/ig/nr-add-nos-generate-profil-table/StructureDefinition-mesures-bundle-flux-alimentation.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-12-11T14:55:17+00:00</t>
+    <t>2023-12-11T15:07:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Bundle du flux d'alimentation à envoyer au serveur</t>
+    <t>Profil de la ressource Bundle du flux d'alimentation à envoyer au serveur</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>